<commit_message>
New Frontend Created and Create Document Updated
</commit_message>
<xml_diff>
--- a/Backend/exports/Documents_Report.xlsx
+++ b/Backend/exports/Documents_Report.xlsx
@@ -11,9 +11,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
-  <si>
-    <t>Document ID</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="39">
+  <si>
+    <t>Srno.</t>
   </si>
   <si>
     <t>Type</t>
@@ -40,6 +40,54 @@
     <t>Billing Info</t>
   </si>
   <si>
+    <t>Inward</t>
+  </si>
+  <si>
+    <t>21/2/2025, 6:09:37 pm</t>
+  </si>
+  <si>
+    <t>LA/0005</t>
+  </si>
+  <si>
+    <t>Internship Offer Latter</t>
+  </si>
+  <si>
+    <t>Dr. Jeegar Trivedi</t>
+  </si>
+  <si>
+    <t>Mr. Bharat  Parmar</t>
+  </si>
+  <si>
+    <t>Received</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>21/2/2025, 3:47:57 am</t>
+  </si>
+  <si>
+    <t>Bill/0001</t>
+  </si>
+  <si>
+    <t>Example Created Document</t>
+  </si>
+  <si>
+    <t>Prof.Apurva Shah</t>
+  </si>
+  <si>
+    <t>18/2/2025, 8:49:51 pm</t>
+  </si>
+  <si>
+    <t>LA/0009</t>
+  </si>
+  <si>
+    <t>Document Reports</t>
+  </si>
+  <si>
+    <t>Dr. Viral  Kapadia</t>
+  </si>
+  <si>
     <t>Outward</t>
   </si>
   <si>
@@ -52,18 +100,6 @@
     <t>Internship Opportunity</t>
   </si>
   <si>
-    <t>Dr. Viral  Kapadia</t>
-  </si>
-  <si>
-    <t>Mr. Bharat  Parmar</t>
-  </si>
-  <si>
-    <t>Received</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>14/2/2025, 10:17:51 pm</t>
   </si>
   <si>
@@ -74,12 +110,6 @@
   </si>
   <si>
     <t>Prof. (Dr.) Apurva Shah</t>
-  </si>
-  <si>
-    <t>Dr. Jeegar Trivedi</t>
-  </si>
-  <si>
-    <t>Inward</t>
   </si>
   <si>
     <t>14/2/2025, 10:05:54 pm</t>
@@ -474,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
@@ -515,7 +545,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -544,7 +574,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -562,7 +592,7 @@
         <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
         <v>15</v>
@@ -573,25 +603,25 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
         <v>22</v>
       </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
+      <c r="F4" t="s">
         <v>24</v>
       </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>21</v>
-      </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
         <v>15</v>
@@ -602,30 +632,117 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
         <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H5" t="s">
         <v>15</v>
       </c>
       <c r="I5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Generate Report by selecting start and end date and get detailed report for the same using backend and frontend part
</commit_message>
<xml_diff>
--- a/Backend/exports/Documents_Report.xlsx
+++ b/Backend/exports/Documents_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
   <si>
     <t>Srno.</t>
   </si>
@@ -43,16 +43,58 @@
     <t>Inward</t>
   </si>
   <si>
-    <t>21/2/2025, 6:09:37 pm</t>
-  </si>
-  <si>
-    <t>LA/0005</t>
-  </si>
-  <si>
-    <t>Internship Offer Latter</t>
-  </si>
-  <si>
-    <t>Dr. Jeegar Trivedi</t>
+    <t>5/3/2025, 2:28:44 pm</t>
+  </si>
+  <si>
+    <t>Installation of openvino</t>
+  </si>
+  <si>
+    <t>Prof. (Dr.) Apurva Shah</t>
+  </si>
+  <si>
+    <t>Mr.Kshitij Gupte</t>
+  </si>
+  <si>
+    <t>Pending Review</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>5/3/2025, 2:24:42 pm</t>
+  </si>
+  <si>
+    <t>Billing of January</t>
+  </si>
+  <si>
+    <t>billing info</t>
+  </si>
+  <si>
+    <t>1/3/2025, 7:37:47 pm</t>
+  </si>
+  <si>
+    <t>JD for Software Engineer</t>
+  </si>
+  <si>
+    <t>Dispatched</t>
+  </si>
+  <si>
+    <t>1/3/2025, 4:32:14 pm</t>
+  </si>
+  <si>
+    <t>What is .NET</t>
+  </si>
+  <si>
+    <t>Outward</t>
+  </si>
+  <si>
+    <t>1/3/2025, 4:27:36 pm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Candidate FAQ </t>
+  </si>
+  <si>
+    <t>Prof.Apurva Shah</t>
   </si>
   <si>
     <t>Mr. Bharat  Parmar</t>
@@ -61,73 +103,7 @@
     <t>Received</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>21/2/2025, 3:47:57 am</t>
-  </si>
-  <si>
-    <t>Bill/0001</t>
-  </si>
-  <si>
-    <t>Example Created Document</t>
-  </si>
-  <si>
-    <t>Prof.Apurva Shah</t>
-  </si>
-  <si>
-    <t>18/2/2025, 8:49:51 pm</t>
-  </si>
-  <si>
-    <t>LA/0009</t>
-  </si>
-  <si>
-    <t>Document Reports</t>
-  </si>
-  <si>
-    <t>Dr. Viral  Kapadia</t>
-  </si>
-  <si>
-    <t>Outward</t>
-  </si>
-  <si>
-    <t>15/2/2025, 3:26:31 pm</t>
-  </si>
-  <si>
-    <t>Circular/0001</t>
-  </si>
-  <si>
-    <t>Internship Opportunity</t>
-  </si>
-  <si>
-    <t>14/2/2025, 10:17:51 pm</t>
-  </si>
-  <si>
-    <t>Notice/0001</t>
-  </si>
-  <si>
-    <t>SS BE-IV Major Project</t>
-  </si>
-  <si>
-    <t>Prof. (Dr.) Apurva Shah</t>
-  </si>
-  <si>
-    <t>14/2/2025, 10:05:54 pm</t>
-  </si>
-  <si>
-    <t>LA/0001</t>
-  </si>
-  <si>
-    <t>Software Developer JD</t>
-  </si>
-  <si>
-    <t>14/2/2025, 9:57:31 pm</t>
-  </si>
-  <si>
-    <t>Student Meeting Record</t>
-  </si>
-  <si>
-    <t>Maheswari Panda</t>
+    <t>not billing</t>
   </si>
 </sst>
 </file>
@@ -504,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
@@ -545,7 +521,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -553,197 +529,124 @@
       <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>15</v>
-      </c>
-      <c r="I2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
       <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
         <v>17</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
         <v>18</v>
-      </c>
-      <c r="E3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
       <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s">
         <v>21</v>
       </c>
-      <c r="D4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>15</v>
-      </c>
-      <c r="I4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
       <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
         <v>15</v>
-      </c>
-      <c r="I5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" t="s">
         <v>29</v>
       </c>
-      <c r="D6" t="s">
+      <c r="I6" t="s">
         <v>30</v>
-      </c>
-      <c r="E6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>1</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Super Admin Dashboard spinner added Analytics component in admin side updated for better user interface and charts graphs updated
Document Report Component updated
Iside the report details
updated

Report Preview Component added now we can view the genarated report before downloading it

Change Password page updated with conent on the page
</commit_message>
<xml_diff>
--- a/Backend/exports/Documents_Report.xlsx
+++ b/Backend/exports/Documents_Report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="176">
   <si>
     <t>Srno.</t>
   </si>
@@ -22,7 +22,7 @@
     <t>DateTime</t>
   </si>
   <si>
-    <t>Letter Serial</t>
+    <t>Document Srno</t>
   </si>
   <si>
     <t>Document Name</t>
@@ -40,28 +40,346 @@
     <t>Billing Info</t>
   </si>
   <si>
+    <t>Outward</t>
+  </si>
+  <si>
+    <t>7/4/2025, 7:12:11 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2025-2026/5</t>
+  </si>
+  <si>
+    <t>INWARD EXAMPLE</t>
+  </si>
+  <si>
+    <t>Prof.Apurva Shah</t>
+  </si>
+  <si>
+    <t>Dr. Jeegar Trivedi</t>
+  </si>
+  <si>
+    <t>Viewed</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>Inward</t>
   </si>
   <si>
+    <t>2/4/2025, 6:41:09 pm</t>
+  </si>
+  <si>
+    <t>COMP/2025-2026/2</t>
+  </si>
+  <si>
+    <t>Billing of 2024-25</t>
+  </si>
+  <si>
+    <t>Prof. (Dr.) Apurva Shah</t>
+  </si>
+  <si>
+    <t>Dr.Kamlesh Vaishnav</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>2/4/2025, 6:34:37 pm</t>
+  </si>
+  <si>
+    <t>COMP/2025-2026/1</t>
+  </si>
+  <si>
+    <t>Holiday Circular</t>
+  </si>
+  <si>
+    <t>Dr. Anjali Jivani</t>
+  </si>
+  <si>
+    <t>2/4/2025, 6:19:45 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2025-2026/1</t>
+  </si>
+  <si>
+    <t>April Document Report</t>
+  </si>
+  <si>
+    <t>Mr. Chaitanya Patel</t>
+  </si>
+  <si>
+    <t>Received</t>
+  </si>
+  <si>
+    <t>27/3/2025, 5:51:22 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/27</t>
+  </si>
+  <si>
+    <t>Internship Offer Letter</t>
+  </si>
+  <si>
+    <t>Pending Review</t>
+  </si>
+  <si>
+    <t>26/3/2025, 9:33:33 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/26</t>
+  </si>
+  <si>
+    <t>Portal Updateed Letter</t>
+  </si>
+  <si>
+    <t>Dr.Hetal Bhavsar</t>
+  </si>
+  <si>
+    <t>26/3/2025, 9:30:29 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/25</t>
+  </si>
+  <si>
+    <t>Billing Document</t>
+  </si>
+  <si>
+    <t>Mr.Kshitij Gupte</t>
+  </si>
+  <si>
+    <t>25/3/2025, 7:11:21 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/24</t>
+  </si>
+  <si>
+    <t>Circular for Maintance</t>
+  </si>
+  <si>
+    <t>21/3/2025, 5:29:02 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/23</t>
+  </si>
+  <si>
+    <t>Document withour rerender</t>
+  </si>
+  <si>
+    <t>20/3/2025, 10:23:57 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/56</t>
+  </si>
+  <si>
+    <t>Notice For Vacation</t>
+  </si>
+  <si>
+    <t>Mr. Bharat  Parmar</t>
+  </si>
+  <si>
+    <t>20/3/2025, 7:21:09 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/55</t>
+  </si>
+  <si>
+    <t>Fest Circular</t>
+  </si>
+  <si>
+    <t>20/3/2025, 7:07:03 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/3</t>
+  </si>
+  <si>
+    <t>Report Generator</t>
+  </si>
+  <si>
+    <t>21/3/2025, 7:41:10 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/22</t>
+  </si>
+  <si>
+    <t>List Of Groups</t>
+  </si>
+  <si>
+    <t>20/3/2025, 6:39:48 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/2</t>
+  </si>
+  <si>
+    <t>Documents Report Feb-Mar</t>
+  </si>
+  <si>
+    <t>20/3/2025, 6:16:13 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/21</t>
+  </si>
+  <si>
+    <t>Summer Internship Offer</t>
+  </si>
+  <si>
+    <t>19/3/2025, 10:25:56 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/20</t>
+  </si>
+  <si>
+    <t>Maintanace Of Computer Centre</t>
+  </si>
+  <si>
+    <t>19/3/2025, 10:15:46 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/19</t>
+  </si>
+  <si>
+    <t>Created Document</t>
+  </si>
+  <si>
+    <t>18/3/2025, 11:18:51 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/46</t>
+  </si>
+  <si>
+    <t>Example Document 3</t>
+  </si>
+  <si>
+    <t>Dr. Viral  Kapadia</t>
+  </si>
+  <si>
+    <t>18/3/2025, 11:11:02 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">January Document Report </t>
+  </si>
+  <si>
+    <t>Maheswari Panda</t>
+  </si>
+  <si>
+    <t>Mrs.Chaitali Bhoi</t>
+  </si>
+  <si>
+    <t>Rejected</t>
+  </si>
+  <si>
+    <t>18/3/2025, 10:02:18 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/1</t>
+  </si>
+  <si>
+    <t>Training Info</t>
+  </si>
+  <si>
+    <t>18/3/2025, 9:59:05 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/17</t>
+  </si>
+  <si>
+    <t>Technical Intern JD</t>
+  </si>
+  <si>
+    <t>18/3/2025, 9:55:22 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/16</t>
+  </si>
+  <si>
+    <t>Evaluation Scheme for Employee</t>
+  </si>
+  <si>
+    <t>18/3/2025, 9:34:09 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/15</t>
+  </si>
+  <si>
+    <t>Student Meeting Records2</t>
+  </si>
+  <si>
+    <t>18/3/2025, 8:47:32 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/39</t>
+  </si>
+  <si>
+    <t>Example Document2</t>
+  </si>
+  <si>
+    <t>15/3/2025, 5:00:34 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/12</t>
+  </si>
+  <si>
+    <t>Employee Records</t>
+  </si>
+  <si>
+    <t>15/3/2025, 4:58:50 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/37</t>
+  </si>
+  <si>
+    <t>Office Report</t>
+  </si>
+  <si>
+    <t>14/3/2025, 4:17:57 am</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/36</t>
+  </si>
+  <si>
+    <t>Odoo Training Opportunity</t>
+  </si>
+  <si>
+    <t>14/3/2025, 12:29:15 am</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/10</t>
+  </si>
+  <si>
+    <t>The sample formate of latterr</t>
+  </si>
+  <si>
+    <t>added billing info in update</t>
+  </si>
+  <si>
+    <t>8/3/2025, 8:54:25 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/9</t>
+  </si>
+  <si>
+    <t>The sample formate of latter</t>
+  </si>
+  <si>
+    <t>Dispatched</t>
+  </si>
+  <si>
     <t>5/3/2025, 2:28:44 pm</t>
   </si>
   <si>
+    <t>COMP/2024-2025/8</t>
+  </si>
+  <si>
     <t>Installation of openvino</t>
   </si>
   <si>
-    <t>Prof. (Dr.) Apurva Shah</t>
-  </si>
-  <si>
-    <t>Mr.Kshitij Gupte</t>
-  </si>
-  <si>
-    <t>Pending Review</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>5/3/2025, 2:24:42 pm</t>
+    <t>17/3/2025, 10:22:12 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/14</t>
   </si>
   <si>
     <t>Billing of January</t>
@@ -73,37 +391,154 @@
     <t>1/3/2025, 7:37:47 pm</t>
   </si>
   <si>
+    <t>COMP/2024-2025/7</t>
+  </si>
+  <si>
     <t>JD for Software Engineer</t>
   </si>
   <si>
-    <t>Dispatched</t>
-  </si>
-  <si>
-    <t>1/3/2025, 4:32:14 pm</t>
-  </si>
-  <si>
-    <t>What is .NET</t>
-  </si>
-  <si>
-    <t>Outward</t>
-  </si>
-  <si>
-    <t>1/3/2025, 4:27:36 pm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Candidate FAQ </t>
-  </si>
-  <si>
-    <t>Prof.Apurva Shah</t>
-  </si>
-  <si>
-    <t>Mr. Bharat  Parmar</t>
-  </si>
-  <si>
-    <t>Received</t>
-  </si>
-  <si>
-    <t>not billing</t>
+    <t>14/3/2025, 3:16:09 am</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/11</t>
+  </si>
+  <si>
+    <t>What is .NET?</t>
+  </si>
+  <si>
+    <t>14/3/2025, 3:20:46 am</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/29</t>
+  </si>
+  <si>
+    <t>Candidate FAQs</t>
+  </si>
+  <si>
+    <t>not billing updated</t>
+  </si>
+  <si>
+    <t>25/2/2025, 9:32:39 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/6</t>
+  </si>
+  <si>
+    <t>AWS Free Tier Acount</t>
+  </si>
+  <si>
+    <t>25/2/2025, 7:49:22 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/27</t>
+  </si>
+  <si>
+    <t>Student Meeting Records</t>
+  </si>
+  <si>
+    <t>23/2/2025, 3:51:00 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/22</t>
+  </si>
+  <si>
+    <t>Example Document</t>
+  </si>
+  <si>
+    <t>21/2/2025, 8:58:49 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/21</t>
+  </si>
+  <si>
+    <t>Code Unnati Marathon</t>
+  </si>
+  <si>
+    <t>21/2/2025, 8:50:08 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/18</t>
+  </si>
+  <si>
+    <t>Spam Email</t>
+  </si>
+  <si>
+    <t>21/2/2025, 8:48:09 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/15</t>
+  </si>
+  <si>
+    <t>21/2/2025, 7:23:59 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/5</t>
+  </si>
+  <si>
+    <t>Intern Offer Latter 2</t>
+  </si>
+  <si>
+    <t>21/2/2025, 6:09:37 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/4</t>
+  </si>
+  <si>
+    <t>Internship Offer Latter</t>
+  </si>
+  <si>
+    <t>21/2/2025, 3:47:57 am</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/3</t>
+  </si>
+  <si>
+    <t>Example Created Document</t>
+  </si>
+  <si>
+    <t>18/2/2025, 8:49:51 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/2</t>
+  </si>
+  <si>
+    <t>Document Reports</t>
+  </si>
+  <si>
+    <t>21/3/2025, 7:52:17 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/5</t>
+  </si>
+  <si>
+    <t>Internship Opportunity</t>
+  </si>
+  <si>
+    <t>14/2/2025, 10:17:51 pm</t>
+  </si>
+  <si>
+    <t>FOTE/2024-2025/4</t>
+  </si>
+  <si>
+    <t>SS BE-IV Major Project</t>
+  </si>
+  <si>
+    <t>17/3/2025, 10:19:47 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/13</t>
+  </si>
+  <si>
+    <t>Software Developer JD</t>
+  </si>
+  <si>
+    <t>14/2/2025, 9:57:31 pm</t>
+  </si>
+  <si>
+    <t>COMP/2024-2025/1</t>
+  </si>
+  <si>
+    <t>Student Meeting Record</t>
   </si>
 </sst>
 </file>
@@ -480,7 +915,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="10" customWidth="1"/>
@@ -521,7 +956,7 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -529,124 +964,1386 @@
       <c r="C2" t="s">
         <v>10</v>
       </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="I3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>31</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="I5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>60</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>59</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>52</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" t="s">
+        <v>62</v>
+      </c>
+      <c r="E14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H14" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>50</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>49</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" t="s">
+        <v>68</v>
+      </c>
+      <c r="E16" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>48</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D17" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" t="s">
+        <v>44</v>
+      </c>
+      <c r="H17" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>47</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>46</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" t="s">
+        <v>79</v>
+      </c>
+      <c r="H19" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>44</v>
+      </c>
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" t="s">
+        <v>82</v>
+      </c>
+      <c r="F20" t="s">
+        <v>83</v>
+      </c>
+      <c r="G20" t="s">
+        <v>84</v>
+      </c>
+      <c r="H20" t="s">
+        <v>85</v>
+      </c>
+      <c r="I20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>43</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" t="s">
+        <v>54</v>
+      </c>
+      <c r="H21" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>84</v>
+      </c>
+      <c r="H22" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>41</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E23" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" t="s">
+        <v>27</v>
+      </c>
+      <c r="H23" t="s">
+        <v>85</v>
+      </c>
+      <c r="I23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>40</v>
+      </c>
+      <c r="B24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" t="s">
+        <v>95</v>
+      </c>
+      <c r="D24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" t="s">
+        <v>97</v>
+      </c>
+      <c r="F24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" t="s">
+        <v>44</v>
+      </c>
+      <c r="H24" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>39</v>
+      </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>98</v>
+      </c>
+      <c r="D25" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" t="s">
+        <v>100</v>
+      </c>
+      <c r="F25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" t="s">
+        <v>54</v>
+      </c>
+      <c r="H25" t="s">
+        <v>15</v>
+      </c>
+      <c r="I25" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>38</v>
+      </c>
+      <c r="B26" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" t="s">
+        <v>101</v>
+      </c>
+      <c r="D26" t="s">
+        <v>102</v>
+      </c>
+      <c r="E26" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" t="s">
+        <v>44</v>
+      </c>
+      <c r="H26" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>37</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>104</v>
+      </c>
+      <c r="D27" t="s">
+        <v>105</v>
+      </c>
+      <c r="E27" t="s">
+        <v>106</v>
+      </c>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" t="s">
+        <v>54</v>
+      </c>
+      <c r="H27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I27" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>36</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>107</v>
+      </c>
+      <c r="D28" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" t="s">
+        <v>54</v>
+      </c>
+      <c r="H28" t="s">
+        <v>15</v>
+      </c>
+      <c r="I28" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>35</v>
+      </c>
+      <c r="B29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" t="s">
+        <v>110</v>
+      </c>
+      <c r="D29" t="s">
+        <v>111</v>
+      </c>
+      <c r="E29" t="s">
+        <v>112</v>
+      </c>
+      <c r="F29" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" t="s">
+        <v>85</v>
+      </c>
+      <c r="I29" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" t="s">
+        <v>114</v>
+      </c>
+      <c r="D30" t="s">
+        <v>115</v>
+      </c>
+      <c r="E30" t="s">
+        <v>116</v>
+      </c>
+      <c r="F30" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" t="s">
+        <v>44</v>
+      </c>
+      <c r="H30" t="s">
+        <v>117</v>
+      </c>
+      <c r="I30" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>33</v>
+      </c>
+      <c r="B31" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" t="s">
+        <v>118</v>
+      </c>
+      <c r="D31" t="s">
+        <v>119</v>
+      </c>
+      <c r="E31" t="s">
+        <v>120</v>
+      </c>
+      <c r="F31" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31" t="s">
+        <v>44</v>
+      </c>
+      <c r="H31" t="s">
+        <v>15</v>
+      </c>
+      <c r="I31" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>32</v>
+      </c>
+      <c r="B32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" t="s">
+        <v>121</v>
+      </c>
+      <c r="D32" t="s">
+        <v>122</v>
+      </c>
+      <c r="E32" t="s">
+        <v>123</v>
+      </c>
+      <c r="F32" t="s">
+        <v>21</v>
+      </c>
+      <c r="G32" t="s">
+        <v>44</v>
+      </c>
+      <c r="H32" t="s">
+        <v>23</v>
+      </c>
+      <c r="I32" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C33" t="s">
+        <v>125</v>
+      </c>
+      <c r="D33" t="s">
+        <v>126</v>
+      </c>
+      <c r="E33" t="s">
+        <v>127</v>
+      </c>
+      <c r="F33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" t="s">
+        <v>44</v>
+      </c>
+      <c r="H33" t="s">
+        <v>15</v>
+      </c>
+      <c r="I33" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>30</v>
+      </c>
+      <c r="B34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" t="s">
+        <v>129</v>
+      </c>
+      <c r="E34" t="s">
+        <v>130</v>
+      </c>
+      <c r="F34" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34" t="s">
+        <v>84</v>
+      </c>
+      <c r="H34" t="s">
+        <v>23</v>
+      </c>
+      <c r="I34" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>29</v>
       </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" t="s">
+        <v>131</v>
+      </c>
+      <c r="D35" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" t="s">
+        <v>133</v>
+      </c>
+      <c r="F35" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" t="s">
+        <v>31</v>
+      </c>
+      <c r="H35" t="s">
+        <v>15</v>
+      </c>
+      <c r="I35" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>28</v>
+      </c>
+      <c r="B36" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" t="s">
+        <v>135</v>
+      </c>
+      <c r="D36" t="s">
+        <v>136</v>
+      </c>
+      <c r="E36" t="s">
+        <v>137</v>
+      </c>
+      <c r="F36" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" t="s">
+        <v>44</v>
+      </c>
+      <c r="H36" t="s">
+        <v>117</v>
+      </c>
+      <c r="I36" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A37">
         <v>27</v>
       </c>
-      <c r="G6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" t="s">
-        <v>30</v>
+      <c r="B37" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>138</v>
+      </c>
+      <c r="D37" t="s">
+        <v>139</v>
+      </c>
+      <c r="E37" t="s">
+        <v>140</v>
+      </c>
+      <c r="F37" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" t="s">
+        <v>54</v>
+      </c>
+      <c r="H37" t="s">
+        <v>15</v>
+      </c>
+      <c r="I37" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>22</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" t="s">
+        <v>141</v>
+      </c>
+      <c r="D38" t="s">
+        <v>142</v>
+      </c>
+      <c r="E38" t="s">
+        <v>143</v>
+      </c>
+      <c r="F38" t="s">
+        <v>84</v>
+      </c>
+      <c r="G38" t="s">
+        <v>22</v>
+      </c>
+      <c r="H38" t="s">
+        <v>15</v>
+      </c>
+      <c r="I38" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>21</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" t="s">
+        <v>144</v>
+      </c>
+      <c r="D39" t="s">
+        <v>145</v>
+      </c>
+      <c r="E39" t="s">
+        <v>146</v>
+      </c>
+      <c r="F39" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" t="s">
+        <v>15</v>
+      </c>
+      <c r="I39" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>18</v>
+      </c>
+      <c r="B40" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" t="s">
+        <v>147</v>
+      </c>
+      <c r="D40" t="s">
+        <v>148</v>
+      </c>
+      <c r="E40" t="s">
+        <v>149</v>
+      </c>
+      <c r="F40" t="s">
+        <v>54</v>
+      </c>
+      <c r="G40" t="s">
+        <v>31</v>
+      </c>
+      <c r="H40" t="s">
+        <v>15</v>
+      </c>
+      <c r="I40" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>15</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
+        <v>150</v>
+      </c>
+      <c r="D41" t="s">
+        <v>151</v>
+      </c>
+      <c r="E41" t="s">
+        <v>149</v>
+      </c>
+      <c r="F41" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" t="s">
+        <v>15</v>
+      </c>
+      <c r="I41" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>14</v>
+      </c>
+      <c r="B42" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" t="s">
+        <v>152</v>
+      </c>
+      <c r="D42" t="s">
+        <v>153</v>
+      </c>
+      <c r="E42" t="s">
+        <v>154</v>
+      </c>
+      <c r="F42" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" t="s">
+        <v>54</v>
+      </c>
+      <c r="H42" t="s">
+        <v>117</v>
+      </c>
+      <c r="I42" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>13</v>
+      </c>
+      <c r="B43" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" t="s">
+        <v>155</v>
+      </c>
+      <c r="D43" t="s">
+        <v>156</v>
+      </c>
+      <c r="E43" t="s">
+        <v>157</v>
+      </c>
+      <c r="F43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>54</v>
+      </c>
+      <c r="H43" t="s">
+        <v>15</v>
+      </c>
+      <c r="I43" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>11</v>
+      </c>
+      <c r="B44" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" t="s">
+        <v>158</v>
+      </c>
+      <c r="D44" t="s">
+        <v>159</v>
+      </c>
+      <c r="E44" t="s">
+        <v>160</v>
+      </c>
+      <c r="F44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" t="s">
+        <v>54</v>
+      </c>
+      <c r="H44" t="s">
+        <v>23</v>
+      </c>
+      <c r="I44" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>10</v>
+      </c>
+      <c r="B45" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" t="s">
+        <v>161</v>
+      </c>
+      <c r="D45" t="s">
+        <v>162</v>
+      </c>
+      <c r="E45" t="s">
+        <v>163</v>
+      </c>
+      <c r="F45" t="s">
+        <v>79</v>
+      </c>
+      <c r="G45" t="s">
+        <v>54</v>
+      </c>
+      <c r="H45" t="s">
+        <v>23</v>
+      </c>
+      <c r="I45" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>9</v>
+      </c>
+      <c r="B46" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" t="s">
+        <v>164</v>
+      </c>
+      <c r="D46" t="s">
+        <v>165</v>
+      </c>
+      <c r="E46" t="s">
+        <v>166</v>
+      </c>
+      <c r="F46" t="s">
+        <v>79</v>
+      </c>
+      <c r="G46" t="s">
+        <v>54</v>
+      </c>
+      <c r="H46" t="s">
+        <v>15</v>
+      </c>
+      <c r="I46" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>8</v>
+      </c>
+      <c r="B47" t="s">
+        <v>9</v>
+      </c>
+      <c r="C47" t="s">
+        <v>167</v>
+      </c>
+      <c r="D47" t="s">
+        <v>168</v>
+      </c>
+      <c r="E47" t="s">
+        <v>169</v>
+      </c>
+      <c r="F47" t="s">
+        <v>21</v>
+      </c>
+      <c r="G47" t="s">
+        <v>14</v>
+      </c>
+      <c r="H47" t="s">
+        <v>15</v>
+      </c>
+      <c r="I47" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>3</v>
+      </c>
+      <c r="B48" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" t="s">
+        <v>170</v>
+      </c>
+      <c r="D48" t="s">
+        <v>171</v>
+      </c>
+      <c r="E48" t="s">
+        <v>172</v>
+      </c>
+      <c r="F48" t="s">
+        <v>14</v>
+      </c>
+      <c r="G48" t="s">
+        <v>79</v>
+      </c>
+      <c r="H48" t="s">
+        <v>15</v>
+      </c>
+      <c r="I48" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>1</v>
+      </c>
+      <c r="B49" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" t="s">
+        <v>173</v>
+      </c>
+      <c r="D49" t="s">
+        <v>174</v>
+      </c>
+      <c r="E49" t="s">
+        <v>175</v>
+      </c>
+      <c r="F49" t="s">
+        <v>83</v>
+      </c>
+      <c r="G49" t="s">
+        <v>14</v>
+      </c>
+      <c r="H49" t="s">
+        <v>85</v>
+      </c>
+      <c r="I49" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>